<commit_message>
Refresh site editorial design and launch readiness
</commit_message>
<xml_diff>
--- a/content/wiki/wiki_topic_editorial_calendar.xlsx
+++ b/content/wiki/wiki_topic_editorial_calendar.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Re8e2e21b4db4459d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Editorial Calendar" sheetId="2" r:id="R6844fd36c5554f54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rbe6c57ede2ad4f1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Editorial Calendar" sheetId="2" r:id="R023d9b3481c24c4e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -233,19 +233,19 @@
     <x:t xml:space="preserve">/wiki/fundraising/liquidation-preferences</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">Bootstrapping vs. Venture Capital</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Comparison</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">bootstrapping-vs-vc</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">/wiki/fundraising/bootstrapping-vs-vc</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">Not Started</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Bootstrapping vs. Venture Capital</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Comparison</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">bootstrapping-vs-vc</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/wiki/fundraising/bootstrapping-vs-vc</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Oversubscribed</x:t>
@@ -1345,7 +1345,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9b9df7effe8e4752"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb6c73ccd0c8d4d91"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1760,7 +1760,7 @@
     <x:mergeCell ref="A19:H21"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe8f9189b8324398"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Radcded8716af49be"/>
 </x:worksheet>
 </file>
 
@@ -2166,8 +2166,8 @@
       <x:c r="J12" s="22" t="s">
         <x:v>73</x:v>
       </x:c>
-      <x:c r="K12" s="20" t="s">
-        <x:v>74</x:v>
+      <x:c r="K12" s="20" t="str">
+        <x:v>Draft Complete</x:v>
       </x:c>
       <x:c r="L12" s="23"/>
     </x:row>
@@ -2192,19 +2192,19 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="G13" s="22" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="H13" s="22" t="s">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="H13" s="22" t="s">
+      <x:c r="I13" s="22" t="s">
         <x:v>76</x:v>
       </x:c>
-      <x:c r="I13" s="22" t="s">
+      <x:c r="J13" s="22" t="s">
         <x:v>77</x:v>
       </x:c>
-      <x:c r="J13" s="22" t="s">
-        <x:v>78</x:v>
-      </x:c>
       <x:c r="K13" s="20" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L13" s="23"/>
     </x:row>
@@ -2241,7 +2241,7 @@
         <x:v>81</x:v>
       </x:c>
       <x:c r="K14" s="20" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L14" s="23"/>
     </x:row>
@@ -2278,7 +2278,7 @@
         <x:v>84</x:v>
       </x:c>
       <x:c r="K15" s="20" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L15" s="23"/>
     </x:row>
@@ -2315,7 +2315,7 @@
         <x:v>87</x:v>
       </x:c>
       <x:c r="K16" s="20" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L16" s="23"/>
     </x:row>
@@ -2352,7 +2352,7 @@
         <x:v>90</x:v>
       </x:c>
       <x:c r="K17" s="20" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L17" s="23"/>
     </x:row>
@@ -2389,7 +2389,7 @@
         <x:v>94</x:v>
       </x:c>
       <x:c r="K18" s="20" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L18" s="23"/>
     </x:row>
@@ -2426,7 +2426,7 @@
         <x:v>97</x:v>
       </x:c>
       <x:c r="K19" s="20" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L19" s="23"/>
     </x:row>
@@ -2463,7 +2463,7 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="K20" s="20" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L20" s="23"/>
     </x:row>
@@ -2500,7 +2500,7 @@
         <x:v>103</x:v>
       </x:c>
       <x:c r="K21" s="20" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L21" s="23"/>
     </x:row>
@@ -2537,7 +2537,7 @@
         <x:v>106</x:v>
       </x:c>
       <x:c r="K22" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L22" s="15"/>
     </x:row>
@@ -2574,7 +2574,7 @@
         <x:v>109</x:v>
       </x:c>
       <x:c r="K23" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L23" s="15"/>
     </x:row>
@@ -2689,7 +2689,7 @@
         <x:v>120</x:v>
       </x:c>
       <x:c r="K26" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L26" s="15"/>
     </x:row>
@@ -2726,7 +2726,7 @@
         <x:v>123</x:v>
       </x:c>
       <x:c r="K27" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L27" s="15"/>
     </x:row>
@@ -2763,7 +2763,7 @@
         <x:v>126</x:v>
       </x:c>
       <x:c r="K28" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L28" s="15"/>
     </x:row>
@@ -2800,7 +2800,7 @@
         <x:v>129</x:v>
       </x:c>
       <x:c r="K29" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L29" s="15"/>
     </x:row>
@@ -2837,7 +2837,7 @@
         <x:v>132</x:v>
       </x:c>
       <x:c r="K30" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L30" s="15"/>
     </x:row>
@@ -2874,7 +2874,7 @@
         <x:v>135</x:v>
       </x:c>
       <x:c r="K31" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L31" s="15"/>
     </x:row>
@@ -2902,7 +2902,7 @@
         <x:v>137</x:v>
       </x:c>
       <x:c r="H32" t="s">
-        <x:v>76</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="I32" t="s">
         <x:v>138</x:v>
@@ -2911,7 +2911,7 @@
         <x:v>139</x:v>
       </x:c>
       <x:c r="K32" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L32" s="15"/>
     </x:row>
@@ -2939,7 +2939,7 @@
         <x:v>140</x:v>
       </x:c>
       <x:c r="H33" t="s">
-        <x:v>76</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="I33" t="s">
         <x:v>141</x:v>
@@ -2948,7 +2948,7 @@
         <x:v>142</x:v>
       </x:c>
       <x:c r="K33" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L33" s="15"/>
     </x:row>
@@ -2985,7 +2985,7 @@
         <x:v>145</x:v>
       </x:c>
       <x:c r="K34" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L34" s="15"/>
     </x:row>
@@ -3022,7 +3022,7 @@
         <x:v>148</x:v>
       </x:c>
       <x:c r="K35" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L35" s="15"/>
     </x:row>
@@ -3059,7 +3059,7 @@
         <x:v>151</x:v>
       </x:c>
       <x:c r="K36" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L36" s="15"/>
     </x:row>
@@ -3096,7 +3096,7 @@
         <x:v>154</x:v>
       </x:c>
       <x:c r="K37" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L37" s="15"/>
     </x:row>
@@ -3124,7 +3124,7 @@
         <x:v>155</x:v>
       </x:c>
       <x:c r="H38" t="s">
-        <x:v>76</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="I38" t="s">
         <x:v>156</x:v>
@@ -3133,7 +3133,7 @@
         <x:v>157</x:v>
       </x:c>
       <x:c r="K38" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L38" s="15"/>
     </x:row>
@@ -3170,7 +3170,7 @@
         <x:v>161</x:v>
       </x:c>
       <x:c r="K39" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L39" s="15"/>
     </x:row>
@@ -3204,7 +3204,7 @@
         <x:v>164</x:v>
       </x:c>
       <x:c r="K40" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L40" s="15"/>
     </x:row>
@@ -3241,7 +3241,7 @@
         <x:v>167</x:v>
       </x:c>
       <x:c r="K41" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L41" s="15" t="s">
         <x:v>168</x:v>
@@ -3280,7 +3280,7 @@
         <x:v>171</x:v>
       </x:c>
       <x:c r="K42" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L42" s="15"/>
     </x:row>
@@ -3317,7 +3317,7 @@
         <x:v>174</x:v>
       </x:c>
       <x:c r="K43" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L43" s="15"/>
     </x:row>
@@ -3354,7 +3354,7 @@
         <x:v>177</x:v>
       </x:c>
       <x:c r="K44" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L44" s="15"/>
     </x:row>
@@ -3391,7 +3391,7 @@
         <x:v>180</x:v>
       </x:c>
       <x:c r="K45" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L45" s="15"/>
     </x:row>
@@ -3428,7 +3428,7 @@
         <x:v>184</x:v>
       </x:c>
       <x:c r="K46" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L46" s="15"/>
     </x:row>
@@ -3465,7 +3465,7 @@
         <x:v>187</x:v>
       </x:c>
       <x:c r="K47" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L47" s="15"/>
     </x:row>
@@ -3502,7 +3502,7 @@
         <x:v>190</x:v>
       </x:c>
       <x:c r="K48" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L48" s="15"/>
     </x:row>
@@ -3539,7 +3539,7 @@
         <x:v>193</x:v>
       </x:c>
       <x:c r="K49" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L49" s="15"/>
     </x:row>
@@ -3576,7 +3576,7 @@
         <x:v>196</x:v>
       </x:c>
       <x:c r="K50" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L50" s="15" t="s">
         <x:v>197</x:v>
@@ -3615,7 +3615,7 @@
         <x:v>200</x:v>
       </x:c>
       <x:c r="K51" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L51" s="15"/>
     </x:row>
@@ -3652,7 +3652,7 @@
         <x:v>203</x:v>
       </x:c>
       <x:c r="K52" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L52" s="15"/>
     </x:row>
@@ -3680,7 +3680,7 @@
         <x:v>205</x:v>
       </x:c>
       <x:c r="H53" t="s">
-        <x:v>76</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="I53" t="s">
         <x:v>206</x:v>
@@ -3689,7 +3689,7 @@
         <x:v>207</x:v>
       </x:c>
       <x:c r="K53" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L53" s="15"/>
     </x:row>
@@ -3726,7 +3726,7 @@
         <x:v>210</x:v>
       </x:c>
       <x:c r="K54" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L54" s="15"/>
     </x:row>
@@ -3763,7 +3763,7 @@
         <x:v>213</x:v>
       </x:c>
       <x:c r="K55" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L55" s="15"/>
     </x:row>
@@ -3800,7 +3800,7 @@
         <x:v>216</x:v>
       </x:c>
       <x:c r="K56" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L56" s="15"/>
     </x:row>
@@ -3837,7 +3837,7 @@
         <x:v>219</x:v>
       </x:c>
       <x:c r="K57" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L57" s="15"/>
     </x:row>
@@ -3874,7 +3874,7 @@
         <x:v>222</x:v>
       </x:c>
       <x:c r="K58" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L58" s="15"/>
     </x:row>
@@ -3911,7 +3911,7 @@
         <x:v>225</x:v>
       </x:c>
       <x:c r="K59" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L59" s="15"/>
     </x:row>
@@ -3939,7 +3939,7 @@
         <x:v>227</x:v>
       </x:c>
       <x:c r="H60" t="s">
-        <x:v>76</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="I60" t="s">
         <x:v>228</x:v>
@@ -3948,7 +3948,7 @@
         <x:v>229</x:v>
       </x:c>
       <x:c r="K60" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L60" s="15"/>
     </x:row>
@@ -3985,7 +3985,7 @@
         <x:v>232</x:v>
       </x:c>
       <x:c r="K61" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L61" s="15"/>
     </x:row>
@@ -4013,7 +4013,7 @@
         <x:v>233</x:v>
       </x:c>
       <x:c r="H62" t="s">
-        <x:v>76</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="I62" t="s">
         <x:v>234</x:v>
@@ -4022,7 +4022,7 @@
         <x:v>235</x:v>
       </x:c>
       <x:c r="K62" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L62" s="15"/>
     </x:row>
@@ -4098,7 +4098,7 @@
         <x:v>240</x:v>
       </x:c>
       <x:c r="K64" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L64" s="15"/>
     </x:row>
@@ -4135,7 +4135,7 @@
         <x:v>243</x:v>
       </x:c>
       <x:c r="K65" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L65" s="15"/>
     </x:row>
@@ -4172,7 +4172,7 @@
         <x:v>246</x:v>
       </x:c>
       <x:c r="K66" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L66" s="15"/>
     </x:row>
@@ -4209,7 +4209,7 @@
         <x:v>250</x:v>
       </x:c>
       <x:c r="K67" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L67" s="15"/>
     </x:row>
@@ -4246,7 +4246,7 @@
         <x:v>253</x:v>
       </x:c>
       <x:c r="K68" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L68" s="15"/>
     </x:row>
@@ -4283,7 +4283,7 @@
         <x:v>256</x:v>
       </x:c>
       <x:c r="K69" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L69" s="15"/>
     </x:row>
@@ -4320,7 +4320,7 @@
         <x:v>259</x:v>
       </x:c>
       <x:c r="K70" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L70" s="15"/>
     </x:row>
@@ -4357,7 +4357,7 @@
         <x:v>262</x:v>
       </x:c>
       <x:c r="K71" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L71" s="15"/>
     </x:row>
@@ -4394,7 +4394,7 @@
         <x:v>265</x:v>
       </x:c>
       <x:c r="K72" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L72" s="15"/>
     </x:row>
@@ -4431,7 +4431,7 @@
         <x:v>268</x:v>
       </x:c>
       <x:c r="K73" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L73" s="15"/>
     </x:row>
@@ -4468,7 +4468,7 @@
         <x:v>272</x:v>
       </x:c>
       <x:c r="K74" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L74" s="15"/>
     </x:row>
@@ -4505,7 +4505,7 @@
         <x:v>275</x:v>
       </x:c>
       <x:c r="K75" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L75" s="15"/>
     </x:row>
@@ -4542,7 +4542,7 @@
         <x:v>278</x:v>
       </x:c>
       <x:c r="K76" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L76" s="15"/>
     </x:row>
@@ -4579,7 +4579,7 @@
         <x:v>281</x:v>
       </x:c>
       <x:c r="K77" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L77" s="15"/>
     </x:row>
@@ -4616,7 +4616,7 @@
         <x:v>284</x:v>
       </x:c>
       <x:c r="K78" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L78" s="15"/>
     </x:row>
@@ -4653,7 +4653,7 @@
         <x:v>287</x:v>
       </x:c>
       <x:c r="K79" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L79" s="15"/>
     </x:row>
@@ -4690,7 +4690,7 @@
         <x:v>290</x:v>
       </x:c>
       <x:c r="K80" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L80" s="15"/>
     </x:row>
@@ -4727,7 +4727,7 @@
         <x:v>294</x:v>
       </x:c>
       <x:c r="K81" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L81" s="15"/>
     </x:row>
@@ -4764,7 +4764,7 @@
         <x:v>297</x:v>
       </x:c>
       <x:c r="K82" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="L82" s="15"/>
     </x:row>
@@ -4806,7 +4806,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra589ffe54a414406"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R131f19c6a7344455"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>